<commit_message>
Actualización automática: 2026-02-24 14:43:38
</commit_message>
<xml_diff>
--- a/Inventory/dynamic_inventory/inventory_data.xlsx
+++ b/Inventory/dynamic_inventory/inventory_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\102627~1\AppData\Roaming\MobaXterm\slash\FTPRemoteFiles\3\0\root@10.181.8.209\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\102627~1\AppData\Roaming\MobaXterm\slash\FTPRemoteFiles\4\0\root@10.181.8.209\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E935998A-7AC4-4542-8FE5-2F8AB7340EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{018785F4-0A4A-4006-8C83-04DBA684261A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="295">
   <si>
     <t>Host</t>
   </si>
@@ -60,12 +60,6 @@
     <t>192.168.97.46</t>
   </si>
   <si>
-    <t>10.181.4.22</t>
-  </si>
-  <si>
-    <t>10.181.4.23</t>
-  </si>
-  <si>
     <t>10.181.4.103</t>
   </si>
   <si>
@@ -165,15 +159,9 @@
     <t>10.181.0.74</t>
   </si>
   <si>
-    <t>10.181.3.148</t>
-  </si>
-  <si>
     <t>10.181.3.156</t>
   </si>
   <si>
-    <t>10.181.3.145</t>
-  </si>
-  <si>
     <t>10.181.3.109</t>
   </si>
   <si>
@@ -186,12 +174,6 @@
     <t xml:space="preserve">alkexadbadm02vm2 </t>
   </si>
   <si>
-    <t>SOA02LNX</t>
-  </si>
-  <si>
-    <t>SOA03LNX</t>
-  </si>
-  <si>
     <t>CRM_BD3_PRD</t>
   </si>
   <si>
@@ -288,13 +270,7 @@
     <t>WS02 - PEOPLESOFT</t>
   </si>
   <si>
-    <t>solsinergiasap</t>
-  </si>
-  <si>
     <t>gspsmsinergia</t>
-  </si>
-  <si>
-    <t>s4sinergiaprd</t>
   </si>
   <si>
     <t>MOVILTRACK</t>
@@ -1292,7 +1268,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F139"/>
+  <dimension ref="A1:F135"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.85546875" customWidth="1"/>
@@ -1319,7 +1295,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1327,13 +1303,13 @@
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>6</v>
@@ -1353,7 +1329,7 @@
         <v>7</v>
       </c>
       <c r="E3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1370,7 +1346,7 @@
         <v>7</v>
       </c>
       <c r="E4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1384,10 +1360,10 @@
         <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>7</v>
+        <v>199</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1404,7 +1380,7 @@
         <v>7</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1421,7 +1397,7 @@
         <v>7</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1437,8 +1413,8 @@
       <c r="D8" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>56</v>
+      <c r="E8" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1454,8 +1430,8 @@
       <c r="D9" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>72</v>
+      <c r="E9" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1471,8 +1447,8 @@
       <c r="D10" t="s">
         <v>7</v>
       </c>
-      <c r="E10" t="s">
-        <v>57</v>
+      <c r="E10" s="3" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1488,8 +1464,8 @@
       <c r="D11" t="s">
         <v>7</v>
       </c>
-      <c r="E11" t="s">
-        <v>58</v>
+      <c r="E11" s="3" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1506,7 +1482,7 @@
         <v>7</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1522,8 +1498,8 @@
       <c r="D13" t="s">
         <v>7</v>
       </c>
-      <c r="E13" s="3" t="s">
-        <v>60</v>
+      <c r="E13" s="4" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1539,8 +1515,11 @@
       <c r="D14" t="s">
         <v>7</v>
       </c>
-      <c r="E14" s="3" t="s">
-        <v>61</v>
+      <c r="E14" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1557,7 +1536,10 @@
         <v>7</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>64</v>
+        <v>56</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1574,10 +1556,10 @@
         <v>7</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1593,11 +1575,11 @@
       <c r="D17" t="s">
         <v>7</v>
       </c>
-      <c r="E17" s="4" t="s">
-        <v>62</v>
+      <c r="E17" t="s">
+        <v>60</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1613,11 +1595,8 @@
       <c r="D18" t="s">
         <v>7</v>
       </c>
-      <c r="E18" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>94</v>
+      <c r="E18" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1634,10 +1613,7 @@
         <v>7</v>
       </c>
       <c r="E19" t="s">
-        <v>66</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>94</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1653,7 +1629,7 @@
       <c r="D20" t="s">
         <v>7</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="3" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1670,8 +1646,8 @@
       <c r="D21" t="s">
         <v>7</v>
       </c>
-      <c r="E21" t="s">
-        <v>68</v>
+      <c r="E21" s="3" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1687,8 +1663,11 @@
       <c r="D22" t="s">
         <v>7</v>
       </c>
-      <c r="E22" s="3" t="s">
-        <v>73</v>
+      <c r="E22" t="s">
+        <v>63</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1705,7 +1684,7 @@
         <v>7</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -1722,10 +1701,7 @@
         <v>7</v>
       </c>
       <c r="E24" t="s">
-        <v>69</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>94</v>
+        <v>68</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -1741,8 +1717,8 @@
       <c r="D25" t="s">
         <v>7</v>
       </c>
-      <c r="E25" s="3" t="s">
-        <v>70</v>
+      <c r="E25" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1759,7 +1735,7 @@
         <v>7</v>
       </c>
       <c r="E26" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1776,7 +1752,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1790,44 +1766,44 @@
         <v>34</v>
       </c>
       <c r="D28" t="s">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="E28" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>36</v>
+      </c>
+      <c r="B29" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" t="s">
+        <v>36</v>
+      </c>
+      <c r="D29" t="s">
         <v>35</v>
       </c>
-      <c r="B29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C29" t="s">
-        <v>35</v>
-      </c>
-      <c r="D29" t="s">
-        <v>7</v>
-      </c>
       <c r="E29" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B30" t="s">
         <v>9</v>
       </c>
       <c r="C30" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D30" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E30" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -1841,10 +1817,10 @@
         <v>38</v>
       </c>
       <c r="D31" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E31" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -1858,13 +1834,13 @@
         <v>39</v>
       </c>
       <c r="D32" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E32" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>40</v>
       </c>
@@ -1875,13 +1851,13 @@
         <v>40</v>
       </c>
       <c r="D33" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E33" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>41</v>
       </c>
@@ -1892,13 +1868,13 @@
         <v>41</v>
       </c>
       <c r="D34" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E34" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>42</v>
       </c>
@@ -1909,13 +1885,13 @@
         <v>42</v>
       </c>
       <c r="D35" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E35" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>43</v>
       </c>
@@ -1926,13 +1902,13 @@
         <v>43</v>
       </c>
       <c r="D36" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E36" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>44</v>
       </c>
@@ -1943,13 +1919,13 @@
         <v>44</v>
       </c>
       <c r="D37" t="s">
-        <v>37</v>
-      </c>
-      <c r="E37" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>45</v>
       </c>
@@ -1960,13 +1936,13 @@
         <v>45</v>
       </c>
       <c r="D38" t="s">
-        <v>37</v>
-      </c>
-      <c r="E38" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>46</v>
       </c>
@@ -1980,92 +1956,86 @@
         <v>7</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="F39" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>88</v>
+      </c>
+      <c r="B40" t="s">
+        <v>89</v>
+      </c>
+      <c r="C40" t="s">
+        <v>88</v>
+      </c>
+      <c r="D40" t="s">
+        <v>7</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B41" t="s">
+        <v>89</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="D41" t="s">
+        <v>7</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="B42" t="s">
+        <v>140</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D42" t="s">
+        <v>7</v>
+      </c>
+      <c r="E42" s="5" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>47</v>
-      </c>
-      <c r="B40" t="s">
-        <v>9</v>
-      </c>
-      <c r="C40" t="s">
-        <v>47</v>
-      </c>
-      <c r="D40" t="s">
-        <v>7</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>48</v>
-      </c>
-      <c r="B41" t="s">
-        <v>9</v>
-      </c>
-      <c r="C41" t="s">
-        <v>48</v>
-      </c>
-      <c r="D41" t="s">
-        <v>7</v>
-      </c>
-      <c r="E41" s="3" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B43" t="s">
         <v>89</v>
       </c>
-      <c r="F41" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>49</v>
-      </c>
-      <c r="B42" t="s">
-        <v>9</v>
-      </c>
-      <c r="C42" t="s">
-        <v>49</v>
-      </c>
-      <c r="D42" t="s">
-        <v>7</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>50</v>
-      </c>
-      <c r="B43" t="s">
-        <v>9</v>
-      </c>
-      <c r="C43" t="s">
-        <v>50</v>
+      <c r="C43" s="5" t="s">
+        <v>95</v>
       </c>
       <c r="D43" t="s">
         <v>7</v>
       </c>
-      <c r="E43" s="3" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+      <c r="E43" s="5" t="s">
         <v>96</v>
       </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
+        <v>97</v>
+      </c>
       <c r="B44" t="s">
+        <v>89</v>
+      </c>
+      <c r="C44" s="5" t="s">
         <v>97</v>
-      </c>
-      <c r="C44" t="s">
-        <v>96</v>
       </c>
       <c r="D44" t="s">
         <v>7</v>
@@ -2074,12 +2044,12 @@
         <v>98</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>99</v>
       </c>
       <c r="B45" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C45" s="5" t="s">
         <v>99</v>
@@ -2091,12 +2061,12 @@
         <v>100</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>101</v>
       </c>
       <c r="B46" t="s">
-        <v>148</v>
+        <v>89</v>
       </c>
       <c r="C46" s="5" t="s">
         <v>101</v>
@@ -2108,12 +2078,12 @@
         <v>102</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>103</v>
       </c>
       <c r="B47" t="s">
-        <v>97</v>
+        <v>140</v>
       </c>
       <c r="C47" s="5" t="s">
         <v>103</v>
@@ -2125,12 +2095,12 @@
         <v>104</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
         <v>105</v>
       </c>
       <c r="B48" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>105</v>
@@ -2147,7 +2117,7 @@
         <v>107</v>
       </c>
       <c r="B49" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>107</v>
@@ -2156,126 +2126,126 @@
         <v>7</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>108</v>
+        <v>141</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B50" t="s">
+        <v>89</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D50" t="s">
+        <v>87</v>
+      </c>
+      <c r="E50" s="5" t="s">
         <v>109</v>
-      </c>
-      <c r="B50" t="s">
-        <v>97</v>
-      </c>
-      <c r="C50" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="D50" t="s">
-        <v>7</v>
-      </c>
-      <c r="E50" s="5" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B51" t="s">
+        <v>140</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="D51" t="s">
+        <v>7</v>
+      </c>
+      <c r="E51" s="5" t="s">
         <v>111</v>
-      </c>
-      <c r="B51" t="s">
-        <v>148</v>
-      </c>
-      <c r="C51" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="D51" t="s">
-        <v>7</v>
-      </c>
-      <c r="E51" s="5" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>113</v>
+        <v>272</v>
       </c>
       <c r="B52" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>113</v>
+        <v>272</v>
       </c>
       <c r="D52" t="s">
-        <v>7</v>
+        <v>87</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>114</v>
+        <v>273</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B53" t="s">
-        <v>97</v>
+        <v>140</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D53" t="s">
         <v>7</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>149</v>
+        <v>113</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B54" t="s">
-        <v>97</v>
+        <v>140</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D54" t="s">
-        <v>95</v>
+        <v>7</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B55" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D55" t="s">
         <v>7</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>280</v>
+        <v>118</v>
       </c>
       <c r="B56" t="s">
-        <v>97</v>
+        <v>140</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>280</v>
+        <v>118</v>
       </c>
       <c r="D56" t="s">
-        <v>95</v>
+        <v>7</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>281</v>
+        <v>119</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
@@ -2283,7 +2253,7 @@
         <v>120</v>
       </c>
       <c r="B57" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C57" s="5" t="s">
         <v>120</v>
@@ -2300,7 +2270,7 @@
         <v>122</v>
       </c>
       <c r="B58" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C58" s="5" t="s">
         <v>122</v>
@@ -2317,7 +2287,7 @@
         <v>124</v>
       </c>
       <c r="B59" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C59" s="5" t="s">
         <v>124</v>
@@ -2334,13 +2304,13 @@
         <v>126</v>
       </c>
       <c r="B60" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C60" s="5" t="s">
         <v>126</v>
       </c>
       <c r="D60" t="s">
-        <v>7</v>
+        <v>87</v>
       </c>
       <c r="E60" s="5" t="s">
         <v>127</v>
@@ -2351,13 +2321,13 @@
         <v>128</v>
       </c>
       <c r="B61" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C61" s="5" t="s">
         <v>128</v>
       </c>
       <c r="D61" t="s">
-        <v>7</v>
+        <v>87</v>
       </c>
       <c r="E61" s="5" t="s">
         <v>129</v>
@@ -2368,47 +2338,47 @@
         <v>130</v>
       </c>
       <c r="B62" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="C62" s="5" t="s">
         <v>130</v>
       </c>
       <c r="D62" t="s">
-        <v>7</v>
+        <v>87</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B63" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D63" t="s">
-        <v>7</v>
+        <v>87</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B64" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D64" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="E64" s="5" t="s">
         <v>135</v>
@@ -2416,1277 +2386,1209 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B65" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D65" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B66" t="s">
+        <v>143</v>
+      </c>
+      <c r="C66" t="s">
+        <v>142</v>
+      </c>
+      <c r="D66" t="s">
+        <v>87</v>
+      </c>
+      <c r="E66" t="s">
         <v>144</v>
       </c>
-      <c r="C66" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="D66" t="s">
-        <v>95</v>
-      </c>
-      <c r="E66" s="5" t="s">
-        <v>141</v>
-      </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" s="5" t="s">
-        <v>139</v>
+      <c r="A67" t="s">
+        <v>260</v>
       </c>
       <c r="B67" t="s">
-        <v>144</v>
-      </c>
-      <c r="C67" s="5" t="s">
-        <v>139</v>
+        <v>200</v>
+      </c>
+      <c r="C67" t="s">
+        <v>260</v>
       </c>
       <c r="D67" t="s">
-        <v>95</v>
-      </c>
-      <c r="E67" s="5" t="s">
-        <v>142</v>
+        <v>199</v>
+      </c>
+      <c r="E67" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="5" t="s">
-        <v>140</v>
+      <c r="A68" t="s">
+        <v>261</v>
       </c>
       <c r="B68" t="s">
-        <v>144</v>
-      </c>
-      <c r="C68" s="5" t="s">
-        <v>140</v>
+        <v>200</v>
+      </c>
+      <c r="C68" t="s">
+        <v>261</v>
       </c>
       <c r="D68" t="s">
-        <v>95</v>
-      </c>
-      <c r="E68" s="5" t="s">
-        <v>143</v>
+        <v>199</v>
+      </c>
+      <c r="E68" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="5" t="s">
-        <v>145</v>
+      <c r="A69" t="s">
+        <v>262</v>
       </c>
       <c r="B69" t="s">
-        <v>146</v>
-      </c>
-      <c r="C69" s="5" t="s">
-        <v>145</v>
+        <v>200</v>
+      </c>
+      <c r="C69" t="s">
+        <v>262</v>
       </c>
       <c r="D69" t="s">
-        <v>95</v>
-      </c>
-      <c r="E69" s="5" t="s">
-        <v>147</v>
+        <v>199</v>
+      </c>
+      <c r="E69" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="5" t="s">
-        <v>150</v>
+      <c r="A70" t="s">
+        <v>263</v>
       </c>
       <c r="B70" t="s">
-        <v>151</v>
+        <v>200</v>
       </c>
       <c r="C70" t="s">
-        <v>150</v>
+        <v>263</v>
       </c>
       <c r="D70" t="s">
-        <v>95</v>
+        <v>199</v>
       </c>
       <c r="E70" t="s">
-        <v>152</v>
+        <v>259</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>268</v>
+        <v>145</v>
       </c>
       <c r="B71" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C71" t="s">
-        <v>268</v>
+        <v>145</v>
       </c>
       <c r="D71" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E71" t="s">
-        <v>264</v>
+        <v>201</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>269</v>
+        <v>146</v>
       </c>
       <c r="B72" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C72" t="s">
-        <v>269</v>
+        <v>146</v>
       </c>
       <c r="D72" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E72" t="s">
-        <v>265</v>
+        <v>202</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>270</v>
+        <v>147</v>
       </c>
       <c r="B73" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C73" t="s">
-        <v>270</v>
+        <v>147</v>
       </c>
       <c r="D73" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E73" t="s">
-        <v>266</v>
+        <v>203</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>271</v>
+        <v>148</v>
       </c>
       <c r="B74" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C74" t="s">
-        <v>271</v>
+        <v>148</v>
       </c>
       <c r="D74" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E74" t="s">
-        <v>267</v>
+        <v>204</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B75" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C75" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="D75" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E75" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B76" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C76" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D76" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E76" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B77" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C77" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D77" t="s">
+        <v>199</v>
+      </c>
+      <c r="E77" t="s">
         <v>207</v>
-      </c>
-      <c r="E77" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B78" t="s">
+        <v>200</v>
+      </c>
+      <c r="C78" t="s">
+        <v>152</v>
+      </c>
+      <c r="D78" t="s">
+        <v>199</v>
+      </c>
+      <c r="E78" t="s">
         <v>208</v>
-      </c>
-      <c r="C78" t="s">
-        <v>156</v>
-      </c>
-      <c r="D78" t="s">
-        <v>207</v>
-      </c>
-      <c r="E78" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B79" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C79" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D79" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E79" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B80" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C80" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="D80" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E80" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B81" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C81" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="D81" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E81" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B82" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C82" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="D82" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E82" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="B83" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C83" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="D83" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E83" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B84" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C84" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="D84" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E84" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B85" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C85" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="D85" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E85" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B86" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C86" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="D86" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E86" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="B87" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C87" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="D87" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E87" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B88" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C88" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D88" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E88" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B89" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C89" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D89" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E89" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B90" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C90" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D90" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E90" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B91" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C91" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="D91" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E91" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B92" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C92" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D92" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E92" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B93" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C93" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="D93" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E93" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B94" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C94" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D94" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E94" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B95" t="s">
-        <v>208</v>
+        <v>266</v>
       </c>
       <c r="C95" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="D95" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E95" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B96" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C96" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D96" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E96" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B97" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C97" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D97" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E97" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B98" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C98" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D98" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E98" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B99" t="s">
-        <v>274</v>
+        <v>200</v>
       </c>
       <c r="C99" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D99" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E99" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B100" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C100" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D100" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E100" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="B101" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C101" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D101" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E101" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B102" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C102" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="D102" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E102" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B103" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C103" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D103" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E103" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B104" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C104" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D104" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E104" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B105" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C105" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D105" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E105" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B106" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C106" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D106" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E106" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B107" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C107" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D107" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E107" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B108" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C108" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D108" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E108" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B109" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C109" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="D109" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E109" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B110" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C110" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D110" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E110" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B111" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C111" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D111" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E111" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B112" t="s">
-        <v>208</v>
+        <v>265</v>
       </c>
       <c r="C112" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D112" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E112" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B113" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C113" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="D113" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E113" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B114" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C114" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D114" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E114" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B115" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C115" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="D115" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E115" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B116" t="s">
-        <v>273</v>
+        <v>200</v>
       </c>
       <c r="C116" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D116" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E116" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="B117" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C117" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="D117" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E117" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="B118" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C118" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D118" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E118" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B119" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C119" t="s">
-        <v>197</v>
+        <v>267</v>
       </c>
       <c r="D119" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E119" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B120" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C120" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D120" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E120" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="B121" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C121" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="D121" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E121" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="B122" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C122" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="D122" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E122" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="B123" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C123" t="s">
-        <v>275</v>
+        <v>197</v>
       </c>
       <c r="D123" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E123" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B124" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C124" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D124" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E124" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
-        <v>203</v>
+      <c r="A125" s="6" t="s">
+        <v>264</v>
       </c>
       <c r="B125" t="s">
-        <v>208</v>
-      </c>
-      <c r="C125" t="s">
-        <v>203</v>
+        <v>200</v>
+      </c>
+      <c r="C125" s="6" t="s">
+        <v>264</v>
       </c>
       <c r="D125" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E125" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>204</v>
+        <v>268</v>
       </c>
       <c r="B126" t="s">
-        <v>208</v>
+        <v>138</v>
       </c>
       <c r="C126" t="s">
-        <v>204</v>
+        <v>268</v>
       </c>
       <c r="D126" t="s">
-        <v>207</v>
+        <v>87</v>
       </c>
       <c r="E126" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>205</v>
+        <v>270</v>
       </c>
       <c r="B127" t="s">
-        <v>208</v>
+        <v>138</v>
       </c>
       <c r="C127" t="s">
-        <v>205</v>
+        <v>270</v>
       </c>
       <c r="D127" t="s">
-        <v>207</v>
+        <v>87</v>
       </c>
       <c r="E127" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>206</v>
+        <v>274</v>
       </c>
       <c r="B128" t="s">
-        <v>208</v>
+        <v>276</v>
       </c>
       <c r="C128" t="s">
-        <v>206</v>
+        <v>274</v>
       </c>
       <c r="D128" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E128" t="s">
-        <v>263</v>
+        <v>275</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A129" s="6" t="s">
-        <v>272</v>
+      <c r="A129" t="s">
+        <v>278</v>
       </c>
       <c r="B129" t="s">
-        <v>208</v>
-      </c>
-      <c r="C129" s="6" t="s">
-        <v>272</v>
+        <v>276</v>
+      </c>
+      <c r="C129" t="s">
+        <v>278</v>
       </c>
       <c r="D129" t="s">
-        <v>207</v>
+        <v>87</v>
       </c>
       <c r="E129" t="s">
-        <v>253</v>
+        <v>277</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
+        <v>279</v>
+      </c>
+      <c r="B130" t="s">
         <v>276</v>
       </c>
-      <c r="B130" t="s">
-        <v>146</v>
-      </c>
       <c r="C130" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="D130" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="E130" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B131" t="s">
-        <v>146</v>
-      </c>
-      <c r="C131" t="s">
-        <v>278</v>
+        <v>282</v>
+      </c>
+      <c r="C131" s="7" t="s">
+        <v>281</v>
       </c>
       <c r="D131" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="E131" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B132" t="s">
+        <v>200</v>
+      </c>
+      <c r="C132" t="s">
         <v>284</v>
       </c>
-      <c r="C132" t="s">
-        <v>282</v>
-      </c>
       <c r="D132" t="s">
-        <v>207</v>
+        <v>87</v>
       </c>
       <c r="E132" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
+        <v>287</v>
+      </c>
+      <c r="B133" t="s">
         <v>286</v>
       </c>
-      <c r="B133" t="s">
-        <v>284</v>
-      </c>
       <c r="C133" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D133" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="E133" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="B134" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="C134" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="D134" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="E134" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B135" t="s">
-        <v>290</v>
-      </c>
-      <c r="C135" s="7" t="s">
-        <v>289</v>
+        <v>293</v>
+      </c>
+      <c r="C135" t="s">
+        <v>292</v>
       </c>
       <c r="D135" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="E135" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A136" t="s">
-        <v>292</v>
-      </c>
-      <c r="B136" t="s">
-        <v>208</v>
-      </c>
-      <c r="C136" t="s">
-        <v>292</v>
-      </c>
-      <c r="D136" t="s">
-        <v>95</v>
-      </c>
-      <c r="E136" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A137" t="s">
-        <v>295</v>
-      </c>
-      <c r="B137" t="s">
         <v>294</v>
-      </c>
-      <c r="C137" t="s">
-        <v>295</v>
-      </c>
-      <c r="D137" t="s">
-        <v>95</v>
-      </c>
-      <c r="E137" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A138" t="s">
-        <v>298</v>
-      </c>
-      <c r="B138" t="s">
-        <v>297</v>
-      </c>
-      <c r="C138" t="s">
-        <v>298</v>
-      </c>
-      <c r="D138" t="s">
-        <v>95</v>
-      </c>
-      <c r="E138" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A139" t="s">
-        <v>300</v>
-      </c>
-      <c r="B139" t="s">
-        <v>301</v>
-      </c>
-      <c r="C139" t="s">
-        <v>300</v>
-      </c>
-      <c r="D139" t="s">
-        <v>95</v>
-      </c>
-      <c r="E139" t="s">
-        <v>302</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática: 2026-04-14 17:12:42
</commit_message>
<xml_diff>
--- a/Inventory/dynamic_inventory/inventory_data.xlsx
+++ b/Inventory/dynamic_inventory/inventory_data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\7167351\AppData\Local\Temp\scp59974\ansible\CIS-Ansible\Inventory\dynamic_inventory\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\7167351\AppData\Local\Temp\scp11124\ansible\CIS-Ansible\Inventory\dynamic_inventory\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95661422-4BDC-4EA5-AD12-5475EAE27A8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61ABB964-9606-4A58-9F2B-121D59ABF680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -910,7 +910,7 @@
     <t>10.181.11.56</t>
   </si>
   <si>
-    <t>pantillaol9</t>
+    <t>plantillaol9</t>
   </si>
 </sst>
 </file>
@@ -1288,13 +1288,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F136"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.08203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1331,7 +1331,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1348,7 +1348,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -1365,7 +1365,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1382,7 +1382,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1399,7 +1399,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1416,7 +1416,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>23</v>
       </c>
@@ -1433,7 +1433,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -1450,7 +1450,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -1467,7 +1467,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>29</v>
       </c>
@@ -1484,7 +1484,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -1501,7 +1501,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>33</v>
       </c>
@@ -1518,7 +1518,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>35</v>
       </c>
@@ -1538,7 +1538,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>38</v>
       </c>
@@ -1558,7 +1558,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>40</v>
       </c>
@@ -1578,7 +1578,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>42</v>
       </c>
@@ -1598,7 +1598,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>44</v>
       </c>
@@ -1615,7 +1615,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>46</v>
       </c>
@@ -1632,7 +1632,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>48</v>
       </c>
@@ -1649,7 +1649,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>50</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>52</v>
       </c>
@@ -1686,7 +1686,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>54</v>
       </c>
@@ -1703,7 +1703,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>56</v>
       </c>
@@ -1720,7 +1720,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>58</v>
       </c>
@@ -1737,7 +1737,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>60</v>
       </c>
@@ -1754,7 +1754,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>62</v>
       </c>
@@ -1771,7 +1771,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>64</v>
       </c>
@@ -1788,7 +1788,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>67</v>
       </c>
@@ -1805,7 +1805,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>69</v>
       </c>
@@ -1822,7 +1822,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>71</v>
       </c>
@@ -1839,7 +1839,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>73</v>
       </c>
@@ -1856,7 +1856,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>75</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>77</v>
       </c>
@@ -1890,7 +1890,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>79</v>
       </c>
@@ -1907,7 +1907,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>81</v>
       </c>
@@ -1924,7 +1924,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>83</v>
       </c>
@@ -1941,7 +1941,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>85</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>87</v>
       </c>
@@ -1975,7 +1975,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>89</v>
       </c>
@@ -1992,7 +1992,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>92</v>
       </c>
@@ -2009,7 +2009,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>94</v>
       </c>
@@ -2026,7 +2026,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>97</v>
       </c>
@@ -2043,7 +2043,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>99</v>
       </c>
@@ -2060,7 +2060,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>101</v>
       </c>
@@ -2077,7 +2077,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>103</v>
       </c>
@@ -2094,7 +2094,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>105</v>
       </c>
@@ -2111,7 +2111,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>107</v>
       </c>
@@ -2128,7 +2128,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>109</v>
       </c>
@@ -2145,7 +2145,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>111</v>
       </c>
@@ -2162,7 +2162,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>113</v>
       </c>
@@ -2179,7 +2179,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>115</v>
       </c>
@@ -2196,7 +2196,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>117</v>
       </c>
@@ -2213,7 +2213,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>119</v>
       </c>
@@ -2230,7 +2230,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>121</v>
       </c>
@@ -2247,7 +2247,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>123</v>
       </c>
@@ -2264,7 +2264,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>125</v>
       </c>
@@ -2281,7 +2281,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>127</v>
       </c>
@@ -2298,7 +2298,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>129</v>
       </c>
@@ -2315,7 +2315,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>131</v>
       </c>
@@ -2332,7 +2332,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="61" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>133</v>
       </c>
@@ -2349,7 +2349,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>135</v>
       </c>
@@ -2366,7 +2366,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="63" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>138</v>
       </c>
@@ -2383,7 +2383,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="64" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>140</v>
       </c>
@@ -2400,7 +2400,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="65" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>142</v>
       </c>
@@ -2417,7 +2417,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="66" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>145</v>
       </c>
@@ -2434,7 +2434,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="67" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>148</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="68" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>151</v>
       </c>
@@ -2468,7 +2468,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="69" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>153</v>
       </c>
@@ -2485,7 +2485,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="70" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>155</v>
       </c>
@@ -2502,7 +2502,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="71" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>157</v>
       </c>
@@ -2519,7 +2519,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="72" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>159</v>
       </c>
@@ -2536,7 +2536,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="73" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>161</v>
       </c>
@@ -2553,7 +2553,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="74" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>163</v>
       </c>
@@ -2570,7 +2570,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="75" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>165</v>
       </c>
@@ -2587,7 +2587,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="76" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>167</v>
       </c>
@@ -2604,7 +2604,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="77" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>169</v>
       </c>
@@ -2621,7 +2621,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="78" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>171</v>
       </c>
@@ -2638,7 +2638,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="79" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>173</v>
       </c>
@@ -2655,7 +2655,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="80" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>175</v>
       </c>
@@ -2672,7 +2672,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="81" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>177</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="82" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>179</v>
       </c>
@@ -2706,7 +2706,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="83" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>181</v>
       </c>
@@ -2723,7 +2723,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="84" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>183</v>
       </c>
@@ -2740,7 +2740,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="85" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>185</v>
       </c>
@@ -2757,7 +2757,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="86" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>187</v>
       </c>
@@ -2774,7 +2774,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="87" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>189</v>
       </c>
@@ -2791,7 +2791,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="88" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>191</v>
       </c>
@@ -2808,7 +2808,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="89" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>193</v>
       </c>
@@ -2825,7 +2825,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="90" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>195</v>
       </c>
@@ -2842,7 +2842,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="91" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>197</v>
       </c>
@@ -2859,7 +2859,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="92" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>199</v>
       </c>
@@ -2876,7 +2876,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="93" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>201</v>
       </c>
@@ -2893,7 +2893,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="94" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>203</v>
       </c>
@@ -2910,7 +2910,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="95" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>205</v>
       </c>
@@ -2927,7 +2927,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="96" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>208</v>
       </c>
@@ -2944,7 +2944,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="97" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>210</v>
       </c>
@@ -2961,7 +2961,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="98" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>212</v>
       </c>
@@ -2978,7 +2978,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="99" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>214</v>
       </c>
@@ -2995,7 +2995,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="100" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>216</v>
       </c>
@@ -3012,7 +3012,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="101" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>218</v>
       </c>
@@ -3029,7 +3029,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="102" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>220</v>
       </c>
@@ -3046,7 +3046,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="103" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>222</v>
       </c>
@@ -3063,7 +3063,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="104" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>224</v>
       </c>
@@ -3080,7 +3080,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="105" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>226</v>
       </c>
@@ -3097,7 +3097,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="106" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>228</v>
       </c>
@@ -3114,7 +3114,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="107" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>230</v>
       </c>
@@ -3131,7 +3131,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="108" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>232</v>
       </c>
@@ -3148,7 +3148,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="109" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>234</v>
       </c>
@@ -3165,7 +3165,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="110" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>236</v>
       </c>
@@ -3182,7 +3182,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="111" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>238</v>
       </c>
@@ -3199,7 +3199,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="112" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>240</v>
       </c>
@@ -3216,7 +3216,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="113" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>243</v>
       </c>
@@ -3233,7 +3233,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="114" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>245</v>
       </c>
@@ -3250,7 +3250,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="115" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>247</v>
       </c>
@@ -3267,7 +3267,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="116" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>249</v>
       </c>
@@ -3284,7 +3284,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="117" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>251</v>
       </c>
@@ -3301,7 +3301,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="118" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>253</v>
       </c>
@@ -3318,7 +3318,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="119" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>255</v>
       </c>
@@ -3335,7 +3335,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="120" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>258</v>
       </c>
@@ -3352,7 +3352,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="121" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>260</v>
       </c>
@@ -3369,7 +3369,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="122" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>262</v>
       </c>
@@ -3386,7 +3386,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="123" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>264</v>
       </c>
@@ -3403,7 +3403,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="124" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>266</v>
       </c>
@@ -3420,7 +3420,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="125" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>268</v>
       </c>
@@ -3437,7 +3437,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="126" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>270</v>
       </c>
@@ -3454,7 +3454,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="127" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>272</v>
       </c>
@@ -3471,7 +3471,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="128" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>274</v>
       </c>
@@ -3488,7 +3488,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="129" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>277</v>
       </c>
@@ -3505,7 +3505,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="130" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>279</v>
       </c>
@@ -3522,7 +3522,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="131" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>281</v>
       </c>
@@ -3539,7 +3539,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="132" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>284</v>
       </c>
@@ -3556,7 +3556,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="133" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>286</v>
       </c>
@@ -3573,7 +3573,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="134" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>289</v>
       </c>
@@ -3590,7 +3590,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="135" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>292</v>
       </c>
@@ -3607,7 +3607,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="136" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>295</v>
       </c>

</xml_diff>